<commit_message>
Initialize Alpha Sense System Alpha v1.0
</commit_message>
<xml_diff>
--- a/03-宏观与周期/债券市场月度跟踪模板/债券市场_月度跟踪_2025-10_11.xlsx
+++ b/03-宏观与周期/债券市场月度跟踪模板/债券市场_月度跟踪_2025-10_11.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eb538877c78419e5/1.文档-积累要看的文件/1. 投资框架/债券市场月度跟踪模板/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eb538877c78419e5/1.积累要看的文件/1. 投资框架/03-宏观与周期/债券市场月度跟踪模板/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_046195969E06338388D7C6F9718B15D0AF041969" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{185134CF-316A-4F37-8FD9-41D9E6ED5BD7}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_046195969E06338388D7C6F9718B15D0AF041969" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73BF888A-6B5C-4A68-ABCE-9CAEF48467ED}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="3157" yWindow="3157" windowWidth="17280" windowHeight="9990" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1833" yWindow="1833" windowWidth="30720" windowHeight="16460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="月度跟踪模板" sheetId="1" r:id="rId1"/>
@@ -684,10 +684,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -976,19 +972,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H38"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.234375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.76171875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.17578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.17578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.05859375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1014,7 +1010,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -1040,7 +1036,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
@@ -1052,7 +1048,7 @@
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
@@ -1064,7 +1060,7 @@
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" s="4" t="s">
         <v>18</v>
       </c>
@@ -1076,7 +1072,7 @@
       <c r="G5" s="5"/>
       <c r="H5" s="5"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
         <v>19</v>
       </c>
@@ -1088,7 +1084,7 @@
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A7" s="4" t="s">
         <v>20</v>
       </c>
@@ -1100,7 +1096,7 @@
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A8" s="4" t="s">
         <v>21</v>
       </c>
@@ -1112,7 +1108,7 @@
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>22</v>
       </c>
@@ -1124,7 +1120,7 @@
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>23</v>
       </c>
@@ -1136,7 +1132,7 @@
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>24</v>
       </c>
@@ -1148,7 +1144,7 @@
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>25</v>
       </c>
@@ -1160,7 +1156,7 @@
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>26</v>
       </c>
@@ -1172,7 +1168,7 @@
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A14" s="4" t="s">
         <v>27</v>
       </c>
@@ -1184,7 +1180,7 @@
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A15" s="4" t="s">
         <v>28</v>
       </c>
@@ -1196,7 +1192,7 @@
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A16" s="4" t="s">
         <v>29</v>
       </c>
@@ -1208,7 +1204,7 @@
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A17" s="4" t="s">
         <v>30</v>
       </c>
@@ -1220,7 +1216,7 @@
       <c r="G17" s="5"/>
       <c r="H17" s="5"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A18" s="4" t="s">
         <v>31</v>
       </c>
@@ -1232,7 +1228,7 @@
       <c r="G18" s="5"/>
       <c r="H18" s="5"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
         <v>32</v>
       </c>
@@ -1244,7 +1240,7 @@
       <c r="G19" s="5"/>
       <c r="H19" s="5"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A20" s="4" t="s">
         <v>33</v>
       </c>
@@ -1256,7 +1252,7 @@
       <c r="G20" s="5"/>
       <c r="H20" s="5"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A21" s="4" t="s">
         <v>34</v>
       </c>
@@ -1268,7 +1264,7 @@
       <c r="G21" s="5"/>
       <c r="H21" s="5"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
         <v>35</v>
       </c>
@@ -1280,7 +1276,7 @@
       <c r="G22" s="5"/>
       <c r="H22" s="5"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A23" s="4" t="s">
         <v>36</v>
       </c>
@@ -1292,7 +1288,7 @@
       <c r="G23" s="5"/>
       <c r="H23" s="5"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A24" s="4" t="s">
         <v>37</v>
       </c>
@@ -1304,7 +1300,7 @@
       <c r="G24" s="5"/>
       <c r="H24" s="5"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A25" s="4" t="s">
         <v>38</v>
       </c>
@@ -1316,7 +1312,7 @@
       <c r="G25" s="5"/>
       <c r="H25" s="5"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
         <v>39</v>
       </c>
@@ -1328,7 +1324,7 @@
       <c r="G26" s="5"/>
       <c r="H26" s="5"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A27" s="4" t="s">
         <v>40</v>
       </c>
@@ -1340,7 +1336,7 @@
       <c r="G27" s="5"/>
       <c r="H27" s="5"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A28" s="4" t="s">
         <v>41</v>
       </c>
@@ -1352,7 +1348,7 @@
       <c r="G28" s="5"/>
       <c r="H28" s="5"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A29" s="4" t="s">
         <v>42</v>
       </c>
@@ -1364,7 +1360,7 @@
       <c r="G29" s="5"/>
       <c r="H29" s="5"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A30" s="4" t="s">
         <v>43</v>
       </c>
@@ -1376,7 +1372,7 @@
       <c r="G30" s="5"/>
       <c r="H30" s="5"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A31" s="4" t="s">
         <v>44</v>
       </c>
@@ -1388,7 +1384,7 @@
       <c r="G31" s="5"/>
       <c r="H31" s="5"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
         <v>45</v>
       </c>
@@ -1400,7 +1396,7 @@
       <c r="G32" s="5"/>
       <c r="H32" s="5"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A33" s="4" t="s">
         <v>46</v>
       </c>
@@ -1412,7 +1408,7 @@
       <c r="G33" s="5"/>
       <c r="H33" s="5"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A34" s="4" t="s">
         <v>47</v>
       </c>
@@ -1424,7 +1420,7 @@
       <c r="G34" s="5"/>
       <c r="H34" s="5"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A35" s="4" t="s">
         <v>48</v>
       </c>
@@ -1436,7 +1432,7 @@
       <c r="G35" s="5"/>
       <c r="H35" s="5"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A36" s="4" t="s">
         <v>49</v>
       </c>
@@ -1448,7 +1444,7 @@
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A37" s="4" t="s">
         <v>50</v>
       </c>
@@ -1460,7 +1456,7 @@
       <c r="G37" s="5"/>
       <c r="H37" s="5"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A38" s="4" t="s">
         <v>51</v>
       </c>
@@ -1501,12 +1497,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="6" width="26" customWidth="1"/>
+    <col min="1" max="1" width="27.46875" customWidth="1"/>
+    <col min="2" max="6" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>1</v>
       </c>
@@ -1526,7 +1523,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>52</v>
       </c>
@@ -1546,7 +1543,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>58</v>
       </c>
@@ -1566,7 +1563,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>64</v>
       </c>
@@ -1586,7 +1583,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>70</v>
       </c>
@@ -1606,7 +1603,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>76</v>
       </c>
@@ -1626,7 +1623,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>82</v>
       </c>
@@ -1646,7 +1643,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>88</v>
       </c>
@@ -1666,7 +1663,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>94</v>
       </c>
@@ -1686,7 +1683,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>100</v>
       </c>
@@ -1706,7 +1703,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>106</v>
       </c>
@@ -1726,7 +1723,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>112</v>
       </c>
@@ -1743,7 +1740,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>117</v>
       </c>
@@ -1760,7 +1757,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>122</v>
       </c>
@@ -1774,7 +1771,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>126</v>
       </c>
@@ -1785,12 +1782,12 @@
         <v>128</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>130</v>
       </c>
@@ -1804,13 +1801,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
         <v>131</v>
       </c>
@@ -1818,7 +1815,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="7" t="s">
         <v>7</v>
       </c>
@@ -1826,7 +1823,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="42" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="7" t="s">
         <v>134</v>
       </c>
@@ -1843,7 +1840,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1855,7 +1852,7 @@
     <col min="8" max="8" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1881,7 +1878,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="74.099999999999994" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="74.099999999999994" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -1907,7 +1904,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="130.1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="9" t="s">
         <v>136</v>
       </c>
@@ -1933,7 +1930,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="130.1" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="9" t="s">
         <v>144</v>
       </c>
@@ -1969,27 +1966,27 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="120" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="8" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="8" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="8" t="s">
         <v>155</v>
       </c>

</xml_diff>